<commit_message>
Update soccer trades 2026-07-28 00:01:21 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Brasileiro Serie B/trades.xlsx
+++ b/data/sxbet/ligas/Brasileiro Serie B/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V26"/>
+  <dimension ref="A1:V35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x92277fd9760c85a724f7658409181352a319dca98f6e6d7257490f3cd59a4395</t>
+          <t>0xabc659ab91438a92bdab313e7d198edb3b35cfb23ca4984e285a9ac861379d39</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,52 +546,52 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2.87432</t>
+          <t>1.44</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.545</t>
+          <t>1.96</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>Brasileiro Serie B</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Sport Club Recife PE 0</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Brasileiro Serie B</t>
-        </is>
-      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE vs Cuiaba</t>
+          <t>CRB vs Vila Nova GO</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>Vila Nova GO</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x3057927dc9e21afe22a23dd6d591a6c725a59b11e00f692f2f923619aca059bc</t>
+          <t>0x5b7e3cab20a9b0ba61a99e9112a570a69a585ccdf9a5378595b25f4a631754f8</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19549019</t>
+          <t>L19549036</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785193206</t>
+          <t>1785196608</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>5.273982</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,31 +643,39 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xff78883ea30011b29c2e39189b8b5fac38d095bfa0dd3b12c2ef9db5a5448c9c</t>
+          <t>0x57d41fa40d47545066168bc258c022eda8e23794c6e8e25f411b7e4dd970bb46</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>0xAB03DDB118c18F7EfC711f056a7A4B5D25e040aA</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>66.47463</t>
+          <t>0.99999</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.7963</t>
+          <t>1.755</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Sport Club Recife PE</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -690,7 +698,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x6b43d60f84d2b8aaad01ff70b0fa90594e13bb82860379b6bf9072320349b0ab</t>
+          <t>0xf919361f092da0369730061828581eef122cbdafb264d98bb5b8de00a91f9f05</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -720,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785193161</t>
+          <t>1785196351</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -730,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>83.484622</t>
+          <t>1.32449</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,7 +755,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x1f877654f3c926ae529b6ddd3c7171b2d13a4a8d5ebf0feacc94d11ce8030cd0</t>
+          <t>0x25cc5a5a3dc674380900ea29d792b1af86c3327ff37f825f3aa224fbcbf44062</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -762,52 +770,52 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>137.93997</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.8975</t>
+          <t>1.9425</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>CRB -0.5</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>Brasileiro Serie B</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Atletico Goianiense</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Brasileiro Serie B</t>
-        </is>
-      </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Atletico Goianiense vs Operario PR</t>
+          <t>CRB vs Vila Nova GO</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Operario PR</t>
+          <t>Vila Nova GO</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xc8ef5bb61583039e96277733cf10bf29a1a696cbdd90f2cb2bccfce1f6069793</t>
+          <t>0xa9304c5be90462f067ad52886159b64d91c9a8468c0aff2fafb714ca682b39e0</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19548984</t>
+          <t>L19549036</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -832,7 +840,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785192985</t>
+          <t>1785195964</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -842,7 +850,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>153.69356</t>
+          <t>1.37931</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,12 +867,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x6430a839f73026cc87b0d5a0b70654fed87b780609d9d10323dbb2e3d5981d2f</t>
+          <t>0x85b409ffce3c34bc2a7a224f3d47f6160bcac6215ac5a26e88aefd1be3e2746b</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0xFD3Cd99B8d9ff9F970d873FD51Db34a241440516</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -874,22 +882,22 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.99998</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.6963</t>
+          <t>1.1887</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Under/Over (5)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Over 5.0</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -899,27 +907,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>CRB vs Vila Nova GO</t>
+          <t>Atletico Goianiense vs Operario PR</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Vila Nova GO</t>
+          <t>Operario PR</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x164012f3264d9ee546eec79c1f187343794314881d9822a8fe97501455cef745</t>
+          <t>0x013806510be87dbff88a95234b44e79f8dfdea721fa2b13058ae7b80918f8f15</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19549036</t>
+          <t>L19548984</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -944,7 +952,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785192506</t>
+          <t>1785195762</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -954,7 +962,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>7.1813</t>
+          <t>7.94702</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,39 +979,31 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xe710e0c0376a72f95ca778f9e5f3a8399edb9a229d58a6de28041cab6ca46ebc</t>
+          <t>0x9d278b56196f77645ec64561ddf9808ae69c1277d4242007e4d1273618a82941</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x9C5e354F1Dd3e2031bE83f341a9FeFdE8739680E</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>52.85</t>
+          <t>8.19999</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>1.9125</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Operario PR</t>
-        </is>
-      </c>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -1011,27 +1011,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Atletico Goianiense vs Operario PR</t>
+          <t>Sport Club Recife PE vs Cuiaba</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>Sport Club Recife PE</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Operario PR</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x009d97ace951d42df767e4f8051070c4ae71bc57b68e13d8724fbd523b67056f</t>
+          <t>0x6b43d60f84d2b8aaad01ff70b0fa90594e13bb82860379b6bf9072320349b0ab</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19548984</t>
+          <t>L19549019</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785191996</t>
+          <t>1785195534</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>587.222222</t>
+          <t>8.98629</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1083,36 +1083,44 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x2dd6170d0bb75ad4506c6e6e7d66349c95078c6af465ead37ce9752e5b0c998b</t>
+          <t>0x14116c881c0f4533487e957da9f15894479617fd313359c0fe53b0fa20817fce</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>66.90021</t>
+          <t>3.39</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.1113</t>
+          <t>1.1713</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
+          <t>Under/Over (5.5)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Over 5.5</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>Brasileiro Serie B</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Brasileiro Serie B</t>
-        </is>
-      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>Atletico Goianiense vs Operario PR</t>
@@ -1130,7 +1138,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0xc8ef5bb61583039e96277733cf10bf29a1a696cbdd90f2cb2bccfce1f6069793</t>
+          <t>0xb3096fc6db0ce08ac34976715534d4d4519e51ff07d5c08d10d24d21f043ed20</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1160,7 +1168,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785191995</t>
+          <t>1785195474</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1170,7 +1178,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>601.350202</t>
+          <t>19.79562</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1187,7 +1195,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x60f51d4feeddc57e7ad54ec8e925642a90b92e40913e7bf9f7d10e2ab8f78f00</t>
+          <t>0xdbcefe6329694816ae2b1cddb39083bd05853147610de44cd9e649e4706bc376</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1195,31 +1203,23 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>342.92992</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.9225</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Under/Over (4.5)</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Over 4.5</t>
-        </is>
-      </c>
+          <t>Under/Over (5)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -1227,27 +1227,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Atletico Goianiense vs Operario PR</t>
+          <t>CRB vs Vila Nova GO</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Operario PR</t>
+          <t>Vila Nova GO</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x563c254290f2bca3349399de0f58716204283212536d68ecebbda660883e8955</t>
+          <t>0x4e6ae57773c8ebdf636c0fd11584596ba79488f311f5684527d05ce8c8349163</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19548984</t>
+          <t>L19549036</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785191869</t>
+          <t>1785194418</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1282,7 +1282,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>6.166667</t>
+          <t>371.739751</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1299,39 +1299,31 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xe778363b4557273dd14de4337865dd189b21126e8ba81bee67f5eb20692ac1c0</t>
+          <t>0xb65013398fea1f959a670b32cb221d15acbf671317155b728665f166550d1ef1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>123.99</t>
+          <t>68.04987</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.5012</t>
+          <t>1.9337</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>CRB -0.5</t>
-        </is>
-      </c>
+          <t>Under/Over (5.5)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -1354,7 +1346,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xa9304c5be90462f067ad52886159b64d91c9a8468c0aff2fafb714ca682b39e0</t>
+          <t>0xa0c82cc27b7148027b5c44487bb49054dc8b7d2cc14542a06b46d9511a59030b</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1384,7 +1376,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785191301</t>
+          <t>1785194417</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1394,7 +1386,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>247.361596</t>
+          <t>72.87804</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1411,28 +1403,28 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x76badc2285724881b122bebddf6b9e6c4c3cf3e4a05d3690b012b1cc148fbfde</t>
+          <t>0x736f6291a00147b17e0499024ccbc920f3d72ee0b45f060fcc31b182c4104a05</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>599.87913</t>
+          <t>377.83</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.7637</t>
+          <t>1.9263</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Under/Over (5.5)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -1458,7 +1450,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xccd12abb617dfc61183a060a3ae6528413e3d3f34e761b9f0acc3557c868245d</t>
+          <t>0xa0c82cc27b7148027b5c44487bb49054dc8b7d2cc14542a06b46d9511a59030b</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1488,7 +1480,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785191158</t>
+          <t>1785194276</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1498,7 +1490,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>785.439123</t>
+          <t>407.91363</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1515,31 +1507,39 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x91ddeba03b208be248ba41a4881c3c4c7d0715d371e6263f2e0b4290cec16b1b</t>
+          <t>0x92277fd9760c85a724f7658409181352a319dca98f6e6d7257490f3cd59a4395</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>49.90293</t>
+          <t>2.87432</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.3813</t>
+          <t>1.545</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
+          <t>Brasileiro Serie B</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Sport Club Recife PE 0</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -1562,7 +1562,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0xd514accb2f809d1aa051e761e590fdb70d8359c432892ab528533d38968148e5</t>
+          <t>0x3057927dc9e21afe22a23dd6d591a6c725a59b11e00f692f2f923619aca059bc</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785191085</t>
+          <t>1785193206</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>130.892931</t>
+          <t>5.273982</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1619,7 +1619,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x5d9ee4415a1e3226e79c82a0ad8402f41a775d58348c69deb79a0f1f8f6795d6</t>
+          <t>0xff78883ea30011b29c2e39189b8b5fac38d095bfa0dd3b12c2ef9db5a5448c9c</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1630,17 +1630,17 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>31.75047</t>
+          <t>66.47463</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.5275</t>
+          <t>1.7963</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -1666,7 +1666,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x54bd394d0f69cdedbefc7e393cac97bba562ca5d9c533011ea99d1ec4c012a2b</t>
+          <t>0x6b43d60f84d2b8aaad01ff70b0fa90594e13bb82860379b6bf9072320349b0ab</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785191085</t>
+          <t>1785193161</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1706,7 +1706,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>60.190464</t>
+          <t>83.484622</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1723,31 +1723,39 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x057b9dc707d522517e9353e2008a44693bea8ac1ca696f3200b57eb2c82453bb</t>
+          <t>0x1f877654f3c926ae529b6ddd3c7171b2d13a4a8d5ebf0feacc94d11ce8030cd0</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>23.10284</t>
+          <t>137.93997</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.3838</t>
+          <t>1.8975</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr"/>
+          <t>Brasileiro Serie B</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Atletico Goianiense</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -1755,27 +1763,27 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE vs Cuiaba</t>
+          <t>Atletico Goianiense vs Operario PR</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>Operario PR</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xd514accb2f809d1aa051e761e590fdb70d8359c432892ab528533d38968148e5</t>
+          <t>0xc8ef5bb61583039e96277733cf10bf29a1a696cbdd90f2cb2bccfce1f6069793</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>L19549019</t>
+          <t>L19548984</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1800,7 +1808,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785191085</t>
+          <t>1785192985</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1810,7 +1818,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>60.20284</t>
+          <t>153.69356</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1827,31 +1835,39 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x6ec8571db656bf4ace15e41ee9319395aaf946ddda18f3df168f286a1a1bb4ff</t>
+          <t>0x6430a839f73026cc87b0d5a0b70654fed87b780609d9d10323dbb2e3d5981d2f</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr"/>
+          <t>0xFD3Cd99B8d9ff9F970d873FD51Db34a241440516</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>8.99</t>
+          <t>4.99998</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.2463</t>
+          <t>1.6963</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -1859,27 +1875,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE vs Cuiaba</t>
+          <t>CRB vs Vila Nova GO</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>Vila Nova GO</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x7f2fb02659d83b890cfe18154671039eb222ef3a24f76c4dc7c26b4868ea21bf</t>
+          <t>0x164012f3264d9ee546eec79c1f187343794314881d9822a8fe97501455cef745</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19549019</t>
+          <t>L19549036</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1904,7 +1920,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785190227</t>
+          <t>1785192506</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1914,7 +1930,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>36.507614</t>
+          <t>7.1813</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1931,7 +1947,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xa9f26cf6e000e4922c2f38b67d28a2deda7559922560443baab526b4b0c61b73</t>
+          <t>0xe710e0c0376a72f95ca778f9e5f3a8399edb9a229d58a6de28041cab6ca46ebc</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1939,51 +1955,59 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>46.73411</t>
+          <t>52.85</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.3313</t>
+          <t>1.09</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Operario PR</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
           <t>Brasileiro Serie B</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Brasileiro Serie B</t>
-        </is>
-      </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>CRB vs Vila Nova GO</t>
+          <t>Atletico Goianiense vs Operario PR</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Vila Nova GO</t>
+          <t>Operario PR</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0xd53171a74e0242d67f30a86b7aaa3d2b2cde7e733a1beb26cf0c703dbab1e0c6</t>
+          <t>0x009d97ace951d42df767e4f8051070c4ae71bc57b68e13d8724fbd523b67056f</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>L19549036</t>
+          <t>L19548984</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2008,7 +2032,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785189680</t>
+          <t>1785191996</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2018,7 +2042,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>141.084106</t>
+          <t>587.222222</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2035,7 +2059,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x0e0907f0172fe7e0b1a15423f1c2ea46f221e75a91330b9fcd0210b43161dffc</t>
+          <t>0x2dd6170d0bb75ad4506c6e6e7d66349c95078c6af465ead37ce9752e5b0c998b</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2046,12 +2070,12 @@
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>70.48505</t>
+          <t>66.90021</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.3313</t>
+          <t>1.1113</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2067,27 +2091,27 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>CRB vs Vila Nova GO</t>
+          <t>Atletico Goianiense vs Operario PR</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Vila Nova GO</t>
+          <t>Operario PR</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0xd53171a74e0242d67f30a86b7aaa3d2b2cde7e733a1beb26cf0c703dbab1e0c6</t>
+          <t>0xc8ef5bb61583039e96277733cf10bf29a1a696cbdd90f2cb2bccfce1f6069793</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>L19549036</t>
+          <t>L19548984</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -2112,7 +2136,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785189678</t>
+          <t>1785191995</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2122,7 +2146,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>212.785057</t>
+          <t>601.350202</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2139,12 +2163,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0xd2e589ce8fd3d5a2041b18219e18e34205c142aa8a4e07e600978a682778f7dd</t>
+          <t>0x60f51d4feeddc57e7ad54ec8e925642a90b92e40913e7bf9f7d10e2ab8f78f00</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2154,22 +2178,22 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>16.03</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.2662</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Under/Over (4.5)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>CRB -1</t>
+          <t>Over 4.5</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2179,27 +2203,27 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>CRB vs Vila Nova GO</t>
+          <t>Atletico Goianiense vs Operario PR</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Vila Nova GO</t>
+          <t>Operario PR</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0xb474c8115d11c43ca774879d23888594610a0050926049c5871c02ad70442828</t>
+          <t>0x563c254290f2bca3349399de0f58716204283212536d68ecebbda660883e8955</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>L19549036</t>
+          <t>L19548984</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2224,7 +2248,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1785189440</t>
+          <t>1785191869</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2234,7 +2258,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>60.206573</t>
+          <t>6.166667</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2251,12 +2275,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x7067e247051a48c87b2711f56e00831cc9cf38c00816148557da5dde43e0b18d</t>
+          <t>0xe778363b4557273dd14de4337865dd189b21126e8ba81bee67f5eb20692ac1c0</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2266,22 +2290,22 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>123.99</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.2312</t>
+          <t>1.5012</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>CRB -0.5</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2291,27 +2315,27 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE vs Cuiaba</t>
+          <t>CRB vs Vila Nova GO</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>Vila Nova GO</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0xcbd93d924a25bfc5eed272e7eebb053f11cd7a088fbde08dafa66b1ccb19d6d2</t>
+          <t>0xa9304c5be90462f067ad52886159b64d91c9a8468c0aff2fafb714ca682b39e0</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>L19549019</t>
+          <t>L19549036</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2336,7 +2360,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1785188684</t>
+          <t>1785191301</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2346,7 +2370,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>5.102703</t>
+          <t>247.361596</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2363,7 +2387,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0xfef3f05953c1b69da0cb3db16102cf296b132ec89570e3b07a5a0c924d4de594</t>
+          <t>0x76badc2285724881b122bebddf6b9e6c4c3cf3e4a05d3690b012b1cc148fbfde</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2371,31 +2395,23 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>15.88</t>
+          <t>599.87913</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.2637</t>
+          <t>1.7637</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>CRB -1</t>
-        </is>
-      </c>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -2418,7 +2434,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0xb474c8115d11c43ca774879d23888594610a0050926049c5871c02ad70442828</t>
+          <t>0xccd12abb617dfc61183a060a3ae6528413e3d3f34e761b9f0acc3557c868245d</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2448,7 +2464,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1785188472</t>
+          <t>1785191158</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2458,7 +2474,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>60.208531</t>
+          <t>785.439123</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2475,39 +2491,31 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0xfc5ef9a86c99fd1897abcd8e09889e7009f6384950e112b87a199335cb42db0a</t>
+          <t>0x91ddeba03b208be248ba41a4881c3c4c7d0715d371e6263f2e0b4290cec16b1b</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0x155C76202e45BE70c50bfeD7eAeA3B98e7716Ff7</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>49.90293</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.3362</t>
+          <t>1.3813</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -2530,7 +2538,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0x8534ef5ad4f16561c7b4121752a6a7b2095d700e69722155902e66e998ff0f55</t>
+          <t>0xd514accb2f809d1aa051e761e590fdb70d8359c432892ab528533d38968148e5</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2560,7 +2568,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1785188354</t>
+          <t>1785191085</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2570,7 +2578,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>2.973978</t>
+          <t>130.892931</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2587,39 +2595,31 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x70f793d7639e9071725b67e5d59645a0ce3151b32e612fa9a3861ddf68c40caa</t>
+          <t>0x5d9ee4415a1e3226e79c82a0ad8402f41a775d58348c69deb79a0f1f8f6795d6</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0x155C76202e45BE70c50bfeD7eAeA3B98e7716Ff7</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>31.75047</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.3362</t>
+          <t>1.5275</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -2642,7 +2642,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0x8534ef5ad4f16561c7b4121752a6a7b2095d700e69722155902e66e998ff0f55</t>
+          <t>0x54bd394d0f69cdedbefc7e393cac97bba562ca5d9c533011ea99d1ec4c012a2b</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1785188354</t>
+          <t>1785191085</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2682,7 +2682,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>2.973978</t>
+          <t>60.190464</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2699,39 +2699,31 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x0b1b494627a939fced86315d5bf47db8fed3489803145f8581ed0e6feeb9778a</t>
+          <t>0x057b9dc707d522517e9353e2008a44693bea8ac1ca696f3200b57eb2c82453bb</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>10.48681</t>
+          <t>23.10284</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.4663</t>
+          <t>1.3838</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Atletico Goianiense</t>
-        </is>
-      </c>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -2739,27 +2731,27 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Atletico Goianiense vs Operario PR</t>
+          <t>Sport Club Recife PE vs Cuiaba</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>Sport Club Recife PE</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Operario PR</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0x12cd5e193bc63289c7fafbc19303377b9c4255fccb0ecd5d041453d8fa88faff</t>
+          <t>0xd514accb2f809d1aa051e761e590fdb70d8359c432892ab528533d38968148e5</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>L19548984</t>
+          <t>L19549019</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2784,7 +2776,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1785188344</t>
+          <t>1785191085</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2794,7 +2786,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>22.491818</t>
+          <t>60.20284</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2811,39 +2803,31 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0xed0c6b1bbdd31be7427b5ffe7a264e0c13f41925ed28604921031109f2b0cefa</t>
+          <t>0x6ec8571db656bf4ace15e41ee9319395aaf946ddda18f3df168f286a1a1bb4ff</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>10.12</t>
+          <t>8.99</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.4575</t>
+          <t>1.2463</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Atletico Goianiense</t>
-        </is>
-      </c>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -2851,27 +2835,27 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Atletico Goianiense vs Operario PR</t>
+          <t>Sport Club Recife PE vs Cuiaba</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>Sport Club Recife PE</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Operario PR</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0x12cd5e193bc63289c7fafbc19303377b9c4255fccb0ecd5d041453d8fa88faff</t>
+          <t>0x7f2fb02659d83b890cfe18154671039eb222ef3a24f76c4dc7c26b4868ea21bf</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>L19548984</t>
+          <t>L19549019</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2896,7 +2880,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1785188299</t>
+          <t>1785190227</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2906,7 +2890,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>22.120219</t>
+          <t>36.507614</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2923,7 +2907,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0x91583f323297c551497af92aef42c1fbe90007daddf717ff653e1533369fe9d5</t>
+          <t>0xa9f26cf6e000e4922c2f38b67d28a2deda7559922560443baab526b4b0c61b73</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2931,31 +2915,23 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
-          <t>16.03</t>
+          <t>46.73411</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.2662</t>
+          <t>1.3313</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>CRB -1</t>
-        </is>
-      </c>
+          <t>Brasileiro Serie B</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -2978,7 +2954,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0xb474c8115d11c43ca774879d23888594610a0050926049c5871c02ad70442828</t>
+          <t>0xd53171a74e0242d67f30a86b7aaa3d2b2cde7e733a1beb26cf0c703dbab1e0c6</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -3008,7 +2984,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1785188207</t>
+          <t>1785189680</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -3018,7 +2994,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>60.206573</t>
+          <t>141.084106</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3035,28 +3011,28 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x093df5c9b7626116d81288cd377d306eb5151086a71a2bd3951894182b307e34</t>
+          <t>0x0e0907f0172fe7e0b1a15423f1c2ea46f221e75a91330b9fcd0210b43161dffc</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0xFBd63A3Adf898EfFf1e5A017f98756dC760eBfb8</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>49.4</t>
+          <t>70.48505</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.7412</t>
+          <t>1.3313</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Brasileiro Serie B</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
@@ -3082,7 +3058,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0xb474c8115d11c43ca774879d23888594610a0050926049c5871c02ad70442828</t>
+          <t>0xd53171a74e0242d67f30a86b7aaa3d2b2cde7e733a1beb26cf0c703dbab1e0c6</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -3112,7 +3088,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1785187880</t>
+          <t>1785189678</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3122,7 +3098,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>66.644182</t>
+          <t>212.785057</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3139,110 +3115,1110 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>0xd2e589ce8fd3d5a2041b18219e18e34205c142aa8a4e07e600978a682778f7dd</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>16.03</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>1.2662</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>CRB -1</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Brasileiro Serie B</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>CRB vs Vila Nova GO</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Vila Nova GO</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>0xb474c8115d11c43ca774879d23888594610a0050926049c5871c02ad70442828</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>L19549036</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>1785189440</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>1785191400</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>60.206573</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>0x7067e247051a48c87b2711f56e00831cc9cf38c00816148557da5dde43e0b18d</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>1.18</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>1.2312</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Cuiaba</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Brasileiro Serie B</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Sport Club Recife PE vs Cuiaba</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Sport Club Recife PE</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Cuiaba</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>0xcbd93d924a25bfc5eed272e7eebb053f11cd7a088fbde08dafa66b1ccb19d6d2</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>L19549019</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>1785188684</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>1785191400</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>5.102703</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>0xfef3f05953c1b69da0cb3db16102cf296b132ec89570e3b07a5a0c924d4de594</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>15.88</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>1.2637</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>CRB -1</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Brasileiro Serie B</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>CRB vs Vila Nova GO</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Vila Nova GO</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>0xb474c8115d11c43ca774879d23888594610a0050926049c5871c02ad70442828</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>L19549036</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>1785188472</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>1785191400</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>60.208531</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>0xfc5ef9a86c99fd1897abcd8e09889e7009f6384950e112b87a199335cb42db0a</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>0x155C76202e45BE70c50bfeD7eAeA3B98e7716Ff7</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>1.3362</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Brasileiro Serie B</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Sport Club Recife PE vs Cuiaba</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Sport Club Recife PE</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Cuiaba</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>0x8534ef5ad4f16561c7b4121752a6a7b2095d700e69722155902e66e998ff0f55</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>L19549019</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>1785188354</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>1785191400</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>2.973978</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>0x70f793d7639e9071725b67e5d59645a0ce3151b32e612fa9a3861ddf68c40caa</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>0x155C76202e45BE70c50bfeD7eAeA3B98e7716Ff7</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>1.3362</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Brasileiro Serie B</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Sport Club Recife PE vs Cuiaba</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Sport Club Recife PE</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Cuiaba</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>0x8534ef5ad4f16561c7b4121752a6a7b2095d700e69722155902e66e998ff0f55</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>L19549019</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>1785188354</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>1785191400</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>2.973978</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>0x0b1b494627a939fced86315d5bf47db8fed3489803145f8581ed0e6feeb9778a</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>10.48681</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>1.4663</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Atletico Goianiense</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Brasileiro Serie B</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Atletico Goianiense vs Operario PR</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Atletico Goianiense</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Operario PR</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>0x12cd5e193bc63289c7fafbc19303377b9c4255fccb0ecd5d041453d8fa88faff</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>L19548984</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>1785188344</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>1785191400</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>22.491818</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>0xed0c6b1bbdd31be7427b5ffe7a264e0c13f41925ed28604921031109f2b0cefa</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>10.12</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>1.4575</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Atletico Goianiense</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Brasileiro Serie B</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Atletico Goianiense vs Operario PR</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Atletico Goianiense</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Operario PR</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>0x12cd5e193bc63289c7fafbc19303377b9c4255fccb0ecd5d041453d8fa88faff</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>L19548984</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>1785188299</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>1785191400</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>22.120219</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>0x91583f323297c551497af92aef42c1fbe90007daddf717ff653e1533369fe9d5</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>16.03</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>1.2662</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>CRB -1</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Brasileiro Serie B</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>CRB vs Vila Nova GO</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Vila Nova GO</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>0xb474c8115d11c43ca774879d23888594610a0050926049c5871c02ad70442828</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>L19549036</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>1785188207</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>1785191400</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>60.206573</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>0x093df5c9b7626116d81288cd377d306eb5151086a71a2bd3951894182b307e34</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>0xFBd63A3Adf898EfFf1e5A017f98756dC760eBfb8</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>49.4</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>1.7412</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Brasileiro Serie B</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>CRB vs Vila Nova GO</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Vila Nova GO</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>0xb474c8115d11c43ca774879d23888594610a0050926049c5871c02ad70442828</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>L19549036</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>1785187880</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>1785191400</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>66.644182</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>0xf90085256f332e2273158e6e0b53485388f9d9e64670022d5b32ffc4aed4b545</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>0xFBd63A3Adf898EfFf1e5A017f98756dC760eBfb8</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
         <is>
           <t>134.62107</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>1.285</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>CRB -1</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H35" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>CRB vs Vila Nova GO</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="J35" t="inlineStr">
         <is>
           <t>CRB</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="K35" t="inlineStr">
         <is>
           <t>Vila Nova GO</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="L35" t="inlineStr">
         <is>
           <t>0xb474c8115d11c43ca774879d23888594610a0050926049c5871c02ad70442828</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="M35" t="inlineStr">
         <is>
           <t>L19549036</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr">
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R26" t="inlineStr">
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
         <is>
           <t>1785187268</t>
         </is>
       </c>
-      <c r="S26" t="inlineStr">
+      <c r="S35" t="inlineStr">
         <is>
           <t>1785191400</t>
         </is>
       </c>
-      <c r="T26" t="inlineStr">
+      <c r="T35" t="inlineStr">
         <is>
           <t>472.354632</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr">
+      <c r="U35" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V26" t="inlineStr">
+      <c r="V35" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-07-28 02:01:12 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Brasileiro Serie B/trades.xlsx
+++ b/data/sxbet/ligas/Brasileiro Serie B/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V35"/>
+  <dimension ref="A1:V36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xabc659ab91438a92bdab313e7d198edb3b35cfb23ca4984e285a9ac861379d39</t>
+          <t>0xb4b479f20b91ce838514c3ba542e267a537f7f7383fb2fb20cc20a34ad087961</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x2B0D772143059220738CEC4818Ff2a1a499c48fD</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,22 +546,22 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.44</t>
+          <t>7.55</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.96</t>
+          <t>1.4725</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -571,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>CRB vs Vila Nova GO</t>
+          <t>Fortaleza vs Botafogo SP</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Vila Nova GO</t>
+          <t>Botafogo SP</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x5b7e3cab20a9b0ba61a99e9112a570a69a585ccdf9a5378595b25f4a631754f8</t>
+          <t>0x3599f80fe106668016172f48bc64e587e98beaa005e69b77cbb5c0a72055b53a</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19549036</t>
+          <t>L19559910</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785196608</t>
+          <t>1785197761</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785191400</t>
+          <t>1785285300</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>15.978836</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,12 +643,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x57d41fa40d47545066168bc258c022eda8e23794c6e8e25f411b7e4dd970bb46</t>
+          <t>0xabc659ab91438a92bdab313e7d198edb3b35cfb23ca4984e285a9ac861379d39</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0xAB03DDB118c18F7EfC711f056a7A4B5D25e040aA</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -658,12 +658,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0.99999</t>
+          <t>1.44</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.755</t>
+          <t>1.96</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -673,7 +673,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -683,27 +683,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE vs Cuiaba</t>
+          <t>CRB vs Vila Nova GO</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>Vila Nova GO</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xf919361f092da0369730061828581eef122cbdafb264d98bb5b8de00a91f9f05</t>
+          <t>0x5b7e3cab20a9b0ba61a99e9112a570a69a585ccdf9a5378595b25f4a631754f8</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19549019</t>
+          <t>L19549036</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785196351</t>
+          <t>1785196608</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1.32449</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,12 +755,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x25cc5a5a3dc674380900ea29d792b1af86c3327ff37f825f3aa224fbcbf44062</t>
+          <t>0x57d41fa40d47545066168bc258c022eda8e23794c6e8e25f411b7e4dd970bb46</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xAB03DDB118c18F7EfC711f056a7A4B5D25e040aA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -770,22 +770,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>0.99999</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.9425</t>
+          <t>1.755</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>CRB -0.5</t>
+          <t>Sport Club Recife PE</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -795,27 +795,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>CRB vs Vila Nova GO</t>
+          <t>Sport Club Recife PE vs Cuiaba</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Sport Club Recife PE</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Vila Nova GO</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xa9304c5be90462f067ad52886159b64d91c9a8468c0aff2fafb714ca682b39e0</t>
+          <t>0xf919361f092da0369730061828581eef122cbdafb264d98bb5b8de00a91f9f05</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19549036</t>
+          <t>L19549019</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785195964</t>
+          <t>1785196351</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1.37931</t>
+          <t>1.32449</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,7 +867,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x85b409ffce3c34bc2a7a224f3d47f6160bcac6215ac5a26e88aefd1be3e2746b</t>
+          <t>0x25cc5a5a3dc674380900ea29d792b1af86c3327ff37f825f3aa224fbcbf44062</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -882,22 +882,22 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.1887</t>
+          <t>1.9425</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Under/Over (5)</t>
+          <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Over 5.0</t>
+          <t>CRB -0.5</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -907,27 +907,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Atletico Goianiense vs Operario PR</t>
+          <t>CRB vs Vila Nova GO</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Operario PR</t>
+          <t>Vila Nova GO</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x013806510be87dbff88a95234b44e79f8dfdea721fa2b13058ae7b80918f8f15</t>
+          <t>0xa9304c5be90462f067ad52886159b64d91c9a8468c0aff2fafb714ca682b39e0</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19548984</t>
+          <t>L19549036</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -952,7 +952,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785195762</t>
+          <t>1785195964</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>7.94702</t>
+          <t>1.37931</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -979,31 +979,39 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x9d278b56196f77645ec64561ddf9808ae69c1277d4242007e4d1273618a82941</t>
+          <t>0x85b409ffce3c34bc2a7a224f3d47f6160bcac6215ac5a26e88aefd1be3e2746b</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x9C5e354F1Dd3e2031bE83f341a9FeFdE8739680E</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.19999</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.9125</t>
+          <t>1.1887</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+          <t>Under/Over (5)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Over 5.0</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -1011,27 +1019,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE vs Cuiaba</t>
+          <t>Atletico Goianiense vs Operario PR</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>Operario PR</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x6b43d60f84d2b8aaad01ff70b0fa90594e13bb82860379b6bf9072320349b0ab</t>
+          <t>0x013806510be87dbff88a95234b44e79f8dfdea721fa2b13058ae7b80918f8f15</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19549019</t>
+          <t>L19548984</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1056,7 +1064,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785195534</t>
+          <t>1785195762</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1066,7 +1074,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>8.98629</t>
+          <t>7.94702</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1083,39 +1091,31 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x14116c881c0f4533487e957da9f15894479617fd313359c0fe53b0fa20817fce</t>
+          <t>0x9d278b56196f77645ec64561ddf9808ae69c1277d4242007e4d1273618a82941</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x9C5e354F1Dd3e2031bE83f341a9FeFdE8739680E</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.39</t>
+          <t>8.19999</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.1713</t>
+          <t>1.9125</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Under/Over (5.5)</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Over 5.5</t>
-        </is>
-      </c>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -1123,27 +1123,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Atletico Goianiense vs Operario PR</t>
+          <t>Sport Club Recife PE vs Cuiaba</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>Sport Club Recife PE</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Operario PR</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0xb3096fc6db0ce08ac34976715534d4d4519e51ff07d5c08d10d24d21f043ed20</t>
+          <t>0x6b43d60f84d2b8aaad01ff70b0fa90594e13bb82860379b6bf9072320349b0ab</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19548984</t>
+          <t>L19549019</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785195474</t>
+          <t>1785195534</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>19.79562</t>
+          <t>8.98629</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1195,7 +1195,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xdbcefe6329694816ae2b1cddb39083bd05853147610de44cd9e649e4706bc376</t>
+          <t>0x14116c881c0f4533487e957da9f15894479617fd313359c0fe53b0fa20817fce</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1203,23 +1203,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>342.92992</t>
+          <t>3.39</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.9225</t>
+          <t>1.1713</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Under/Over (5)</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
+          <t>Under/Over (5.5)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Over 5.5</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -1227,27 +1235,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>CRB vs Vila Nova GO</t>
+          <t>Atletico Goianiense vs Operario PR</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Vila Nova GO</t>
+          <t>Operario PR</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x4e6ae57773c8ebdf636c0fd11584596ba79488f311f5684527d05ce8c8349163</t>
+          <t>0xb3096fc6db0ce08ac34976715534d4d4519e51ff07d5c08d10d24d21f043ed20</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19549036</t>
+          <t>L19548984</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1272,7 +1280,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785194418</t>
+          <t>1785195474</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1282,7 +1290,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>371.739751</t>
+          <t>19.79562</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1299,7 +1307,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xb65013398fea1f959a670b32cb221d15acbf671317155b728665f166550d1ef1</t>
+          <t>0xdbcefe6329694816ae2b1cddb39083bd05853147610de44cd9e649e4706bc376</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1310,17 +1318,17 @@
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>68.04987</t>
+          <t>342.92992</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.9337</t>
+          <t>1.9225</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Under/Over (5.5)</t>
+          <t>Under/Over (5)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -1346,7 +1354,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xa0c82cc27b7148027b5c44487bb49054dc8b7d2cc14542a06b46d9511a59030b</t>
+          <t>0x4e6ae57773c8ebdf636c0fd11584596ba79488f311f5684527d05ce8c8349163</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1376,7 +1384,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785194417</t>
+          <t>1785194418</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1386,7 +1394,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>72.87804</t>
+          <t>371.739751</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1403,7 +1411,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x736f6291a00147b17e0499024ccbc920f3d72ee0b45f060fcc31b182c4104a05</t>
+          <t>0xb65013398fea1f959a670b32cb221d15acbf671317155b728665f166550d1ef1</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1414,12 +1422,12 @@
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>377.83</t>
+          <t>68.04987</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.9263</t>
+          <t>1.9337</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1480,7 +1488,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785194276</t>
+          <t>1785194417</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1490,7 +1498,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>407.91363</t>
+          <t>72.87804</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1507,67 +1515,59 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x92277fd9760c85a724f7658409181352a319dca98f6e6d7257490f3cd59a4395</t>
+          <t>0x736f6291a00147b17e0499024ccbc920f3d72ee0b45f060fcc31b182c4104a05</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2.87432</t>
+          <t>377.83</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.545</t>
+          <t>1.9263</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
+          <t>Under/Over (5.5)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
           <t>Brasileiro Serie B</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Sport Club Recife PE 0</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Brasileiro Serie B</t>
-        </is>
-      </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE vs Cuiaba</t>
+          <t>CRB vs Vila Nova GO</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>Vila Nova GO</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x3057927dc9e21afe22a23dd6d591a6c725a59b11e00f692f2f923619aca059bc</t>
+          <t>0xa0c82cc27b7148027b5c44487bb49054dc8b7d2cc14542a06b46d9511a59030b</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>L19549019</t>
+          <t>L19549036</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785193206</t>
+          <t>1785194276</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>5.273982</t>
+          <t>407.91363</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1619,31 +1619,39 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xff78883ea30011b29c2e39189b8b5fac38d095bfa0dd3b12c2ef9db5a5448c9c</t>
+          <t>0x92277fd9760c85a724f7658409181352a319dca98f6e6d7257490f3cd59a4395</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>66.47463</t>
+          <t>2.87432</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.7963</t>
+          <t>1.545</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
+          <t>Brasileiro Serie B</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Sport Club Recife PE 0</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -1666,7 +1674,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x6b43d60f84d2b8aaad01ff70b0fa90594e13bb82860379b6bf9072320349b0ab</t>
+          <t>0x3057927dc9e21afe22a23dd6d591a6c725a59b11e00f692f2f923619aca059bc</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1696,7 +1704,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785193161</t>
+          <t>1785193206</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1706,7 +1714,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>83.484622</t>
+          <t>5.273982</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1723,67 +1731,59 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x1f877654f3c926ae529b6ddd3c7171b2d13a4a8d5ebf0feacc94d11ce8030cd0</t>
+          <t>0xff78883ea30011b29c2e39189b8b5fac38d095bfa0dd3b12c2ef9db5a5448c9c</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>137.93997</t>
+          <t>66.47463</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.8975</t>
+          <t>1.7963</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
           <t>Brasileiro Serie B</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Atletico Goianiense</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Brasileiro Serie B</t>
-        </is>
-      </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Atletico Goianiense vs Operario PR</t>
+          <t>Sport Club Recife PE vs Cuiaba</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>Sport Club Recife PE</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Operario PR</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xc8ef5bb61583039e96277733cf10bf29a1a696cbdd90f2cb2bccfce1f6069793</t>
+          <t>0x6b43d60f84d2b8aaad01ff70b0fa90594e13bb82860379b6bf9072320349b0ab</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>L19548984</t>
+          <t>L19549019</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785192985</t>
+          <t>1785193161</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1818,7 +1818,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>153.69356</t>
+          <t>83.484622</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1835,12 +1835,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x6430a839f73026cc87b0d5a0b70654fed87b780609d9d10323dbb2e3d5981d2f</t>
+          <t>0x1f877654f3c926ae529b6ddd3c7171b2d13a4a8d5ebf0feacc94d11ce8030cd0</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0xFD3Cd99B8d9ff9F970d873FD51Db34a241440516</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1850,22 +1850,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>4.99998</t>
+          <t>137.93997</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.6963</t>
+          <t>1.8975</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Brasileiro Serie B</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1875,27 +1875,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>CRB vs Vila Nova GO</t>
+          <t>Atletico Goianiense vs Operario PR</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Vila Nova GO</t>
+          <t>Operario PR</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x164012f3264d9ee546eec79c1f187343794314881d9822a8fe97501455cef745</t>
+          <t>0xc8ef5bb61583039e96277733cf10bf29a1a696cbdd90f2cb2bccfce1f6069793</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19549036</t>
+          <t>L19548984</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785192506</t>
+          <t>1785192985</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1930,7 +1930,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>7.1813</t>
+          <t>153.69356</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1947,12 +1947,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xe710e0c0376a72f95ca778f9e5f3a8399edb9a229d58a6de28041cab6ca46ebc</t>
+          <t>0x6430a839f73026cc87b0d5a0b70654fed87b780609d9d10323dbb2e3d5981d2f</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3Cd99B8d9ff9F970d873FD51Db34a241440516</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1962,22 +1962,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>52.85</t>
+          <t>4.99998</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>1.6963</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Operario PR</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1987,27 +1987,27 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Atletico Goianiense vs Operario PR</t>
+          <t>CRB vs Vila Nova GO</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Operario PR</t>
+          <t>Vila Nova GO</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x009d97ace951d42df767e4f8051070c4ae71bc57b68e13d8724fbd523b67056f</t>
+          <t>0x164012f3264d9ee546eec79c1f187343794314881d9822a8fe97501455cef745</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>L19548984</t>
+          <t>L19549036</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785191996</t>
+          <t>1785192506</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2042,7 +2042,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>587.222222</t>
+          <t>7.1813</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2059,7 +2059,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x2dd6170d0bb75ad4506c6e6e7d66349c95078c6af465ead37ce9752e5b0c998b</t>
+          <t>0xe710e0c0376a72f95ca778f9e5f3a8399edb9a229d58a6de28041cab6ca46ebc</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2067,28 +2067,36 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>66.90021</t>
+          <t>52.85</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.1113</t>
+          <t>1.09</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Operario PR</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
           <t>Brasileiro Serie B</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Brasileiro Serie B</t>
-        </is>
-      </c>
       <c r="I16" t="inlineStr">
         <is>
           <t>Atletico Goianiense vs Operario PR</t>
@@ -2106,7 +2114,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0xc8ef5bb61583039e96277733cf10bf29a1a696cbdd90f2cb2bccfce1f6069793</t>
+          <t>0x009d97ace951d42df767e4f8051070c4ae71bc57b68e13d8724fbd523b67056f</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2136,7 +2144,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785191995</t>
+          <t>1785191996</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2146,7 +2154,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>601.350202</t>
+          <t>587.222222</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2163,39 +2171,31 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x60f51d4feeddc57e7ad54ec8e925642a90b92e40913e7bf9f7d10e2ab8f78f00</t>
+          <t>0x2dd6170d0bb75ad4506c6e6e7d66349c95078c6af465ead37ce9752e5b0c998b</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>66.90021</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.1113</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Under/Over (4.5)</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Over 4.5</t>
-        </is>
-      </c>
+          <t>Brasileiro Serie B</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -2218,7 +2218,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x563c254290f2bca3349399de0f58716204283212536d68ecebbda660883e8955</t>
+          <t>0xc8ef5bb61583039e96277733cf10bf29a1a696cbdd90f2cb2bccfce1f6069793</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2248,7 +2248,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1785191869</t>
+          <t>1785191995</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>6.166667</t>
+          <t>601.350202</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2275,12 +2275,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0xe778363b4557273dd14de4337865dd189b21126e8ba81bee67f5eb20692ac1c0</t>
+          <t>0x60f51d4feeddc57e7ad54ec8e925642a90b92e40913e7bf9f7d10e2ab8f78f00</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2290,22 +2290,22 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>123.99</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.5012</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>Under/Over (4.5)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>CRB -0.5</t>
+          <t>Over 4.5</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2315,27 +2315,27 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>CRB vs Vila Nova GO</t>
+          <t>Atletico Goianiense vs Operario PR</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Vila Nova GO</t>
+          <t>Operario PR</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0xa9304c5be90462f067ad52886159b64d91c9a8468c0aff2fafb714ca682b39e0</t>
+          <t>0x563c254290f2bca3349399de0f58716204283212536d68ecebbda660883e8955</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>L19549036</t>
+          <t>L19548984</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2360,7 +2360,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1785191301</t>
+          <t>1785191869</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2370,7 +2370,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>247.361596</t>
+          <t>6.166667</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2387,31 +2387,39 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x76badc2285724881b122bebddf6b9e6c4c3cf3e4a05d3690b012b1cc148fbfde</t>
+          <t>0xe778363b4557273dd14de4337865dd189b21126e8ba81bee67f5eb20692ac1c0</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
+          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>599.87913</t>
+          <t>123.99</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.7637</t>
+          <t>1.5012</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>CRB -0.5</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -2434,7 +2442,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0xccd12abb617dfc61183a060a3ae6528413e3d3f34e761b9f0acc3557c868245d</t>
+          <t>0xa9304c5be90462f067ad52886159b64d91c9a8468c0aff2fafb714ca682b39e0</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2464,7 +2472,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1785191158</t>
+          <t>1785191301</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2474,7 +2482,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>785.439123</t>
+          <t>247.361596</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2491,7 +2499,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x91ddeba03b208be248ba41a4881c3c4c7d0715d371e6263f2e0b4290cec16b1b</t>
+          <t>0x76badc2285724881b122bebddf6b9e6c4c3cf3e4a05d3690b012b1cc148fbfde</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2502,17 +2510,17 @@
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>49.90293</t>
+          <t>599.87913</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.3813</t>
+          <t>1.7637</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
@@ -2523,27 +2531,27 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE vs Cuiaba</t>
+          <t>CRB vs Vila Nova GO</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>Vila Nova GO</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0xd514accb2f809d1aa051e761e590fdb70d8359c432892ab528533d38968148e5</t>
+          <t>0xccd12abb617dfc61183a060a3ae6528413e3d3f34e761b9f0acc3557c868245d</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>L19549019</t>
+          <t>L19549036</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -2568,7 +2576,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1785191085</t>
+          <t>1785191158</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2578,7 +2586,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>130.892931</t>
+          <t>785.439123</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2595,7 +2603,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x5d9ee4415a1e3226e79c82a0ad8402f41a775d58348c69deb79a0f1f8f6795d6</t>
+          <t>0x91ddeba03b208be248ba41a4881c3c4c7d0715d371e6263f2e0b4290cec16b1b</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2606,17 +2614,17 @@
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>31.75047</t>
+          <t>49.90293</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.5275</t>
+          <t>1.3813</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
@@ -2642,7 +2650,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0x54bd394d0f69cdedbefc7e393cac97bba562ca5d9c533011ea99d1ec4c012a2b</t>
+          <t>0xd514accb2f809d1aa051e761e590fdb70d8359c432892ab528533d38968148e5</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2682,7 +2690,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>60.190464</t>
+          <t>130.892931</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2699,7 +2707,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x057b9dc707d522517e9353e2008a44693bea8ac1ca696f3200b57eb2c82453bb</t>
+          <t>0x5d9ee4415a1e3226e79c82a0ad8402f41a775d58348c69deb79a0f1f8f6795d6</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2710,17 +2718,17 @@
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>23.10284</t>
+          <t>31.75047</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.3838</t>
+          <t>1.5275</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -2746,7 +2754,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0xd514accb2f809d1aa051e761e590fdb70d8359c432892ab528533d38968148e5</t>
+          <t>0x54bd394d0f69cdedbefc7e393cac97bba562ca5d9c533011ea99d1ec4c012a2b</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2786,7 +2794,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>60.20284</t>
+          <t>60.190464</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2803,28 +2811,28 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x6ec8571db656bf4ace15e41ee9319395aaf946ddda18f3df168f286a1a1bb4ff</t>
+          <t>0x057b9dc707d522517e9353e2008a44693bea8ac1ca696f3200b57eb2c82453bb</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>8.99</t>
+          <t>23.10284</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.2463</t>
+          <t>1.3838</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
@@ -2850,7 +2858,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0x7f2fb02659d83b890cfe18154671039eb222ef3a24f76c4dc7c26b4868ea21bf</t>
+          <t>0xd514accb2f809d1aa051e761e590fdb70d8359c432892ab528533d38968148e5</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2880,7 +2888,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1785190227</t>
+          <t>1785191085</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2890,7 +2898,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>36.507614</t>
+          <t>60.20284</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2907,28 +2915,28 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0xa9f26cf6e000e4922c2f38b67d28a2deda7559922560443baab526b4b0c61b73</t>
+          <t>0x6ec8571db656bf4ace15e41ee9319395aaf946ddda18f3df168f286a1a1bb4ff</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
-          <t>46.73411</t>
+          <t>8.99</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.3313</t>
+          <t>1.2463</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Brasileiro Serie B</t>
+          <t>Asian Handicap (0.5)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
@@ -2939,27 +2947,27 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>CRB vs Vila Nova GO</t>
+          <t>Sport Club Recife PE vs Cuiaba</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Sport Club Recife PE</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Vila Nova GO</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0xd53171a74e0242d67f30a86b7aaa3d2b2cde7e733a1beb26cf0c703dbab1e0c6</t>
+          <t>0x7f2fb02659d83b890cfe18154671039eb222ef3a24f76c4dc7c26b4868ea21bf</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>L19549036</t>
+          <t>L19549019</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2984,7 +2992,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1785189680</t>
+          <t>1785190227</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -2994,7 +3002,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>141.084106</t>
+          <t>36.507614</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3011,7 +3019,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x0e0907f0172fe7e0b1a15423f1c2ea46f221e75a91330b9fcd0210b43161dffc</t>
+          <t>0xa9f26cf6e000e4922c2f38b67d28a2deda7559922560443baab526b4b0c61b73</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3022,7 +3030,7 @@
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>70.48505</t>
+          <t>46.73411</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -3088,7 +3096,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1785189678</t>
+          <t>1785189680</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3098,7 +3106,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>212.785057</t>
+          <t>141.084106</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3115,7 +3123,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0xd2e589ce8fd3d5a2041b18219e18e34205c142aa8a4e07e600978a682778f7dd</t>
+          <t>0x0e0907f0172fe7e0b1a15423f1c2ea46f221e75a91330b9fcd0210b43161dffc</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3123,31 +3131,23 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>16.03</t>
+          <t>70.48505</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.2662</t>
+          <t>1.3313</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>CRB -1</t>
-        </is>
-      </c>
+          <t>Brasileiro Serie B</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -3170,7 +3170,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0xb474c8115d11c43ca774879d23888594610a0050926049c5871c02ad70442828</t>
+          <t>0xd53171a74e0242d67f30a86b7aaa3d2b2cde7e733a1beb26cf0c703dbab1e0c6</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3200,7 +3200,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1785189440</t>
+          <t>1785189678</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>60.206573</t>
+          <t>212.785057</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3227,12 +3227,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x7067e247051a48c87b2711f56e00831cc9cf38c00816148557da5dde43e0b18d</t>
+          <t>0xd2e589ce8fd3d5a2041b18219e18e34205c142aa8a4e07e600978a682778f7dd</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -3242,22 +3242,22 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>16.03</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.2312</t>
+          <t>1.2662</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>CRB -1</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3267,27 +3267,27 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE vs Cuiaba</t>
+          <t>CRB vs Vila Nova GO</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>Vila Nova GO</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0xcbd93d924a25bfc5eed272e7eebb053f11cd7a088fbde08dafa66b1ccb19d6d2</t>
+          <t>0xb474c8115d11c43ca774879d23888594610a0050926049c5871c02ad70442828</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>L19549019</t>
+          <t>L19549036</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -3312,7 +3312,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1785188684</t>
+          <t>1785189440</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3322,7 +3322,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>5.102703</t>
+          <t>60.206573</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3339,12 +3339,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0xfef3f05953c1b69da0cb3db16102cf296b132ec89570e3b07a5a0c924d4de594</t>
+          <t>0x7067e247051a48c87b2711f56e00831cc9cf38c00816148557da5dde43e0b18d</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -3354,22 +3354,22 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>15.88</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.2637</t>
+          <t>1.2312</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>CRB -1</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -3379,27 +3379,27 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>CRB vs Vila Nova GO</t>
+          <t>Sport Club Recife PE vs Cuiaba</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Sport Club Recife PE</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Vila Nova GO</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0xb474c8115d11c43ca774879d23888594610a0050926049c5871c02ad70442828</t>
+          <t>0xcbd93d924a25bfc5eed272e7eebb053f11cd7a088fbde08dafa66b1ccb19d6d2</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>L19549036</t>
+          <t>L19549019</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -3424,7 +3424,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1785188472</t>
+          <t>1785188684</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3434,7 +3434,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>60.208531</t>
+          <t>5.102703</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3451,12 +3451,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0xfc5ef9a86c99fd1897abcd8e09889e7009f6384950e112b87a199335cb42db0a</t>
+          <t>0xfef3f05953c1b69da0cb3db16102cf296b132ec89570e3b07a5a0c924d4de594</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>0x155C76202e45BE70c50bfeD7eAeA3B98e7716Ff7</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -3466,22 +3466,22 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15.88</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.3362</t>
+          <t>1.2637</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>CRB -1</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -3491,27 +3491,27 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE vs Cuiaba</t>
+          <t>CRB vs Vila Nova GO</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>Vila Nova GO</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0x8534ef5ad4f16561c7b4121752a6a7b2095d700e69722155902e66e998ff0f55</t>
+          <t>0xb474c8115d11c43ca774879d23888594610a0050926049c5871c02ad70442828</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>L19549019</t>
+          <t>L19549036</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -3536,7 +3536,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1785188354</t>
+          <t>1785188472</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3546,7 +3546,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>2.973978</t>
+          <t>60.208531</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3563,7 +3563,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0x70f793d7639e9071725b67e5d59645a0ce3151b32e612fa9a3861ddf68c40caa</t>
+          <t>0xfc5ef9a86c99fd1897abcd8e09889e7009f6384950e112b87a199335cb42db0a</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3675,12 +3675,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0x0b1b494627a939fced86315d5bf47db8fed3489803145f8581ed0e6feeb9778a</t>
+          <t>0x70f793d7639e9071725b67e5d59645a0ce3151b32e612fa9a3861ddf68c40caa</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x155C76202e45BE70c50bfeD7eAeA3B98e7716Ff7</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -3690,12 +3690,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>10.48681</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.4663</t>
+          <t>1.3362</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3705,7 +3705,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -3715,27 +3715,27 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Atletico Goianiense vs Operario PR</t>
+          <t>Sport Club Recife PE vs Cuiaba</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>Sport Club Recife PE</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Operario PR</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0x12cd5e193bc63289c7fafbc19303377b9c4255fccb0ecd5d041453d8fa88faff</t>
+          <t>0x8534ef5ad4f16561c7b4121752a6a7b2095d700e69722155902e66e998ff0f55</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>L19548984</t>
+          <t>L19549019</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -3760,7 +3760,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1785188344</t>
+          <t>1785188354</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -3770,7 +3770,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>22.491818</t>
+          <t>2.973978</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3787,7 +3787,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0xed0c6b1bbdd31be7427b5ffe7a264e0c13f41925ed28604921031109f2b0cefa</t>
+          <t>0x0b1b494627a939fced86315d5bf47db8fed3489803145f8581ed0e6feeb9778a</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3802,12 +3802,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>10.12</t>
+          <t>10.48681</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.4575</t>
+          <t>1.4663</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3872,7 +3872,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1785188299</t>
+          <t>1785188344</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3882,7 +3882,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>22.120219</t>
+          <t>22.491818</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3899,12 +3899,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0x91583f323297c551497af92aef42c1fbe90007daddf717ff653e1533369fe9d5</t>
+          <t>0xed0c6b1bbdd31be7427b5ffe7a264e0c13f41925ed28604921031109f2b0cefa</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -3914,22 +3914,22 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>16.03</t>
+          <t>10.12</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.2662</t>
+          <t>1.4575</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>CRB -1</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -3939,27 +3939,27 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>CRB vs Vila Nova GO</t>
+          <t>Atletico Goianiense vs Operario PR</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Vila Nova GO</t>
+          <t>Operario PR</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>0xb474c8115d11c43ca774879d23888594610a0050926049c5871c02ad70442828</t>
+          <t>0x12cd5e193bc63289c7fafbc19303377b9c4255fccb0ecd5d041453d8fa88faff</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>L19549036</t>
+          <t>L19548984</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1785188207</t>
+          <t>1785188299</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -3994,7 +3994,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>60.206573</t>
+          <t>22.120219</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4011,23 +4011,27 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0x093df5c9b7626116d81288cd377d306eb5151086a71a2bd3951894182b307e34</t>
+          <t>0x91583f323297c551497af92aef42c1fbe90007daddf717ff653e1533369fe9d5</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>0xFBd63A3Adf898EfFf1e5A017f98756dC760eBfb8</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>49.4</t>
+          <t>16.03</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.7412</t>
+          <t>1.2662</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4035,7 +4039,11 @@
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>CRB -1</t>
+        </is>
+      </c>
       <c r="H34" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -4088,7 +4096,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1785187880</t>
+          <t>1785188207</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -4098,7 +4106,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>66.644182</t>
+          <t>60.206573</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4115,110 +4123,214 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>0x093df5c9b7626116d81288cd377d306eb5151086a71a2bd3951894182b307e34</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>0xFBd63A3Adf898EfFf1e5A017f98756dC760eBfb8</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>49.4</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>1.7412</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Brasileiro Serie B</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>CRB vs Vila Nova GO</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Vila Nova GO</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>0xb474c8115d11c43ca774879d23888594610a0050926049c5871c02ad70442828</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>L19549036</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>1785187880</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>1785191400</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>66.644182</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>0xf90085256f332e2273158e6e0b53485388f9d9e64670022d5b32ffc4aed4b545</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>0xFBd63A3Adf898EfFf1e5A017f98756dC760eBfb8</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
         <is>
           <t>134.62107</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>1.285</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="G36" t="inlineStr">
         <is>
           <t>CRB -1</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="H36" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>CRB vs Vila Nova GO</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="J36" t="inlineStr">
         <is>
           <t>CRB</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
+      <c r="K36" t="inlineStr">
         <is>
           <t>Vila Nova GO</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr">
+      <c r="L36" t="inlineStr">
         <is>
           <t>0xb474c8115d11c43ca774879d23888594610a0050926049c5871c02ad70442828</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr">
+      <c r="M36" t="inlineStr">
         <is>
           <t>L19549036</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P35" t="inlineStr">
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R35" t="inlineStr">
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
         <is>
           <t>1785187268</t>
         </is>
       </c>
-      <c r="S35" t="inlineStr">
+      <c r="S36" t="inlineStr">
         <is>
           <t>1785191400</t>
         </is>
       </c>
-      <c r="T35" t="inlineStr">
+      <c r="T36" t="inlineStr">
         <is>
           <t>472.354632</t>
         </is>
       </c>
-      <c r="U35" t="inlineStr">
+      <c r="U36" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V35" t="inlineStr">
+      <c r="V36" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-07-28 13:01:10 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Brasileiro Serie B/trades.xlsx
+++ b/data/sxbet/ligas/Brasileiro Serie B/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V38"/>
+  <dimension ref="A1:V39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,28 +531,28 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x85007358e98dbb990331e0d5e03719f7274a06e30a530f113f1fc85f8dae9d5e</t>
+          <t>0x134ce73e5e5de4ec678fbc24d939fd1c23d93fecc469eaad9f0912ea8215807e</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xa141274f45d09C2533035cd3c6ab42F3470dF7A8</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>17.81999</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.4775</t>
+          <t>1.695</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -563,27 +563,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Fortaleza vs Botafogo SP</t>
+          <t>EC Juventude RS vs Avai FC SC</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>EC Juventude RS</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Botafogo SP</t>
+          <t>Avai FC SC</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x959c25c0728cb401efff0d745ea009b6084680d22430e206eaee06ed55a415f2</t>
+          <t>0x054a718341f697906bd5b90b8e2d7c7f543f045edf28d7906162f62d38bc2e89</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19559910</t>
+          <t>L19559167</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +608,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785236871</t>
+          <t>1785242761</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785285300</t>
+          <t>1785277800</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>272.251309</t>
+          <t>25.640273</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,23 +635,23 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x97d70935bf599335fadeabf7fc6eb753eed562cb72e0f89e5e87aa178d838696</t>
+          <t>0x85007358e98dbb990331e0d5e03719f7274a06e30a530f113f1fc85f8dae9d5e</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
+          <t>0xa141274f45d09C2533035cd3c6ab42F3470dF7A8</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1.03</t>
+          <t>130</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.5162</t>
+          <t>1.4775</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -667,27 +667,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Ponte Preta vs Athletic Club MG</t>
+          <t>Fortaleza vs Botafogo SP</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Ponte Preta</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Athletic Club MG</t>
+          <t>Botafogo SP</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x5752b3d95bf8e8653ea407ba3c202901e039d83b9c2a96b7932125d7d136bbaf</t>
+          <t>0x959c25c0728cb401efff0d745ea009b6084680d22430e206eaee06ed55a415f2</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19559225</t>
+          <t>L19559910</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -712,17 +712,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785235017</t>
+          <t>1785236871</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1785277800</t>
+          <t>1785285300</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1.995157</t>
+          <t>272.251309</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -739,39 +739,31 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xb4b479f20b91ce838514c3ba542e267a537f7f7383fb2fb20cc20a34ad087961</t>
+          <t>0x97d70935bf599335fadeabf7fc6eb753eed562cb72e0f89e5e87aa178d838696</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x2B0D772143059220738CEC4818Ff2a1a499c48fD</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.55</t>
+          <t>1.03</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.4725</t>
+          <t>1.5162</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -779,27 +771,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Fortaleza vs Botafogo SP</t>
+          <t>Ponte Preta vs Athletic Club MG</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Ponte Preta</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Botafogo SP</t>
+          <t>Athletic Club MG</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x3599f80fe106668016172f48bc64e587e98beaa005e69b77cbb5c0a72055b53a</t>
+          <t>0x5752b3d95bf8e8653ea407ba3c202901e039d83b9c2a96b7932125d7d136bbaf</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19559910</t>
+          <t>L19559225</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -824,17 +816,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785197761</t>
+          <t>1785235017</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1785285300</t>
+          <t>1785277800</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>15.978836</t>
+          <t>1.995157</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -851,12 +843,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xabc659ab91438a92bdab313e7d198edb3b35cfb23ca4984e285a9ac861379d39</t>
+          <t>0xb4b479f20b91ce838514c3ba542e267a537f7f7383fb2fb20cc20a34ad087961</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x2B0D772143059220738CEC4818Ff2a1a499c48fD</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -866,22 +858,22 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1.44</t>
+          <t>7.55</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.96</t>
+          <t>1.4725</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -891,27 +883,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>CRB vs Vila Nova GO</t>
+          <t>Fortaleza vs Botafogo SP</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Vila Nova GO</t>
+          <t>Botafogo SP</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x5b7e3cab20a9b0ba61a99e9112a570a69a585ccdf9a5378595b25f4a631754f8</t>
+          <t>0x3599f80fe106668016172f48bc64e587e98beaa005e69b77cbb5c0a72055b53a</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19549036</t>
+          <t>L19559910</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -936,17 +928,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785196608</t>
+          <t>1785197761</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1785191400</t>
+          <t>1785285300</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>15.978836</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -963,12 +955,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x57d41fa40d47545066168bc258c022eda8e23794c6e8e25f411b7e4dd970bb46</t>
+          <t>0xabc659ab91438a92bdab313e7d198edb3b35cfb23ca4984e285a9ac861379d39</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0xAB03DDB118c18F7EfC711f056a7A4B5D25e040aA</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -978,12 +970,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.99999</t>
+          <t>1.44</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.755</t>
+          <t>1.96</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -993,7 +985,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1003,27 +995,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE vs Cuiaba</t>
+          <t>CRB vs Vila Nova GO</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>Vila Nova GO</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xf919361f092da0369730061828581eef122cbdafb264d98bb5b8de00a91f9f05</t>
+          <t>0x5b7e3cab20a9b0ba61a99e9112a570a69a585ccdf9a5378595b25f4a631754f8</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19549019</t>
+          <t>L19549036</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1048,7 +1040,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785196351</t>
+          <t>1785196608</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1058,7 +1050,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1.32449</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1075,12 +1067,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x25cc5a5a3dc674380900ea29d792b1af86c3327ff37f825f3aa224fbcbf44062</t>
+          <t>0x57d41fa40d47545066168bc258c022eda8e23794c6e8e25f411b7e4dd970bb46</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xAB03DDB118c18F7EfC711f056a7A4B5D25e040aA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1090,22 +1082,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>0.99999</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.9425</t>
+          <t>1.755</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>CRB -0.5</t>
+          <t>Sport Club Recife PE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1115,27 +1107,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>CRB vs Vila Nova GO</t>
+          <t>Sport Club Recife PE vs Cuiaba</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Sport Club Recife PE</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Vila Nova GO</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0xa9304c5be90462f067ad52886159b64d91c9a8468c0aff2fafb714ca682b39e0</t>
+          <t>0xf919361f092da0369730061828581eef122cbdafb264d98bb5b8de00a91f9f05</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19549036</t>
+          <t>L19549019</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1160,7 +1152,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785195964</t>
+          <t>1785196351</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1170,7 +1162,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1.37931</t>
+          <t>1.32449</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1187,7 +1179,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x85b409ffce3c34bc2a7a224f3d47f6160bcac6215ac5a26e88aefd1be3e2746b</t>
+          <t>0x25cc5a5a3dc674380900ea29d792b1af86c3327ff37f825f3aa224fbcbf44062</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1202,22 +1194,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.1887</t>
+          <t>1.9425</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Under/Over (5)</t>
+          <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Over 5.0</t>
+          <t>CRB -0.5</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1227,27 +1219,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Atletico Goianiense vs Operario PR</t>
+          <t>CRB vs Vila Nova GO</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Operario PR</t>
+          <t>Vila Nova GO</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x013806510be87dbff88a95234b44e79f8dfdea721fa2b13058ae7b80918f8f15</t>
+          <t>0xa9304c5be90462f067ad52886159b64d91c9a8468c0aff2fafb714ca682b39e0</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19548984</t>
+          <t>L19549036</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1272,7 +1264,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785195762</t>
+          <t>1785195964</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1282,7 +1274,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>7.94702</t>
+          <t>1.37931</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1299,31 +1291,39 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x9d278b56196f77645ec64561ddf9808ae69c1277d4242007e4d1273618a82941</t>
+          <t>0x85b409ffce3c34bc2a7a224f3d47f6160bcac6215ac5a26e88aefd1be3e2746b</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x9C5e354F1Dd3e2031bE83f341a9FeFdE8739680E</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>8.19999</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.9125</t>
+          <t>1.1887</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
+          <t>Under/Over (5)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Over 5.0</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -1331,27 +1331,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE vs Cuiaba</t>
+          <t>Atletico Goianiense vs Operario PR</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>Operario PR</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x6b43d60f84d2b8aaad01ff70b0fa90594e13bb82860379b6bf9072320349b0ab</t>
+          <t>0x013806510be87dbff88a95234b44e79f8dfdea721fa2b13058ae7b80918f8f15</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19549019</t>
+          <t>L19548984</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1376,7 +1376,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785195534</t>
+          <t>1785195762</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>8.98629</t>
+          <t>7.94702</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1403,39 +1403,31 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x14116c881c0f4533487e957da9f15894479617fd313359c0fe53b0fa20817fce</t>
+          <t>0x9d278b56196f77645ec64561ddf9808ae69c1277d4242007e4d1273618a82941</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x9C5e354F1Dd3e2031bE83f341a9FeFdE8739680E</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3.39</t>
+          <t>8.19999</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.1713</t>
+          <t>1.9125</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Under/Over (5.5)</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Over 5.5</t>
-        </is>
-      </c>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -1443,27 +1435,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Atletico Goianiense vs Operario PR</t>
+          <t>Sport Club Recife PE vs Cuiaba</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>Sport Club Recife PE</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Operario PR</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xb3096fc6db0ce08ac34976715534d4d4519e51ff07d5c08d10d24d21f043ed20</t>
+          <t>0x6b43d60f84d2b8aaad01ff70b0fa90594e13bb82860379b6bf9072320349b0ab</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19548984</t>
+          <t>L19549019</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1488,7 +1480,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785195474</t>
+          <t>1785195534</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1498,7 +1490,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>19.79562</t>
+          <t>8.98629</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1515,7 +1507,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xdbcefe6329694816ae2b1cddb39083bd05853147610de44cd9e649e4706bc376</t>
+          <t>0x14116c881c0f4533487e957da9f15894479617fd313359c0fe53b0fa20817fce</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1523,23 +1515,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>342.92992</t>
+          <t>3.39</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.9225</t>
+          <t>1.1713</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Under/Over (5)</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
+          <t>Under/Over (5.5)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Over 5.5</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -1547,27 +1547,27 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>CRB vs Vila Nova GO</t>
+          <t>Atletico Goianiense vs Operario PR</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Vila Nova GO</t>
+          <t>Operario PR</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x4e6ae57773c8ebdf636c0fd11584596ba79488f311f5684527d05ce8c8349163</t>
+          <t>0xb3096fc6db0ce08ac34976715534d4d4519e51ff07d5c08d10d24d21f043ed20</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>L19549036</t>
+          <t>L19548984</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785194418</t>
+          <t>1785195474</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>371.739751</t>
+          <t>19.79562</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1619,7 +1619,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xb65013398fea1f959a670b32cb221d15acbf671317155b728665f166550d1ef1</t>
+          <t>0xdbcefe6329694816ae2b1cddb39083bd05853147610de44cd9e649e4706bc376</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1630,17 +1630,17 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>68.04987</t>
+          <t>342.92992</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.9337</t>
+          <t>1.9225</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Under/Over (5.5)</t>
+          <t>Under/Over (5)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -1666,7 +1666,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0xa0c82cc27b7148027b5c44487bb49054dc8b7d2cc14542a06b46d9511a59030b</t>
+          <t>0x4e6ae57773c8ebdf636c0fd11584596ba79488f311f5684527d05ce8c8349163</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785194417</t>
+          <t>1785194418</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1706,7 +1706,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>72.87804</t>
+          <t>371.739751</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1723,7 +1723,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x736f6291a00147b17e0499024ccbc920f3d72ee0b45f060fcc31b182c4104a05</t>
+          <t>0xb65013398fea1f959a670b32cb221d15acbf671317155b728665f166550d1ef1</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1734,12 +1734,12 @@
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>377.83</t>
+          <t>68.04987</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.9263</t>
+          <t>1.9337</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1800,7 +1800,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785194276</t>
+          <t>1785194417</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>407.91363</t>
+          <t>72.87804</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1827,67 +1827,59 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x92277fd9760c85a724f7658409181352a319dca98f6e6d7257490f3cd59a4395</t>
+          <t>0x736f6291a00147b17e0499024ccbc920f3d72ee0b45f060fcc31b182c4104a05</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2.87432</t>
+          <t>377.83</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.545</t>
+          <t>1.9263</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
+          <t>Under/Over (5.5)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
           <t>Brasileiro Serie B</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Sport Club Recife PE 0</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Brasileiro Serie B</t>
-        </is>
-      </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE vs Cuiaba</t>
+          <t>CRB vs Vila Nova GO</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>Vila Nova GO</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x3057927dc9e21afe22a23dd6d591a6c725a59b11e00f692f2f923619aca059bc</t>
+          <t>0xa0c82cc27b7148027b5c44487bb49054dc8b7d2cc14542a06b46d9511a59030b</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19549019</t>
+          <t>L19549036</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1912,7 +1904,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785193206</t>
+          <t>1785194276</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1922,7 +1914,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>5.273982</t>
+          <t>407.91363</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1939,31 +1931,39 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xff78883ea30011b29c2e39189b8b5fac38d095bfa0dd3b12c2ef9db5a5448c9c</t>
+          <t>0x92277fd9760c85a724f7658409181352a319dca98f6e6d7257490f3cd59a4395</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>66.47463</t>
+          <t>2.87432</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.7963</t>
+          <t>1.545</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr"/>
+          <t>Brasileiro Serie B</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Sport Club Recife PE 0</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x6b43d60f84d2b8aaad01ff70b0fa90594e13bb82860379b6bf9072320349b0ab</t>
+          <t>0x3057927dc9e21afe22a23dd6d591a6c725a59b11e00f692f2f923619aca059bc</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2016,7 +2016,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785193161</t>
+          <t>1785193206</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>83.484622</t>
+          <t>5.273982</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2043,67 +2043,59 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x1f877654f3c926ae529b6ddd3c7171b2d13a4a8d5ebf0feacc94d11ce8030cd0</t>
+          <t>0xff78883ea30011b29c2e39189b8b5fac38d095bfa0dd3b12c2ef9db5a5448c9c</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>137.93997</t>
+          <t>66.47463</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.8975</t>
+          <t>1.7963</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
           <t>Brasileiro Serie B</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Atletico Goianiense</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Brasileiro Serie B</t>
-        </is>
-      </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Atletico Goianiense vs Operario PR</t>
+          <t>Sport Club Recife PE vs Cuiaba</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>Sport Club Recife PE</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Operario PR</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0xc8ef5bb61583039e96277733cf10bf29a1a696cbdd90f2cb2bccfce1f6069793</t>
+          <t>0x6b43d60f84d2b8aaad01ff70b0fa90594e13bb82860379b6bf9072320349b0ab</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>L19548984</t>
+          <t>L19549019</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -2128,7 +2120,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785192985</t>
+          <t>1785193161</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2138,7 +2130,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>153.69356</t>
+          <t>83.484622</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2155,12 +2147,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x6430a839f73026cc87b0d5a0b70654fed87b780609d9d10323dbb2e3d5981d2f</t>
+          <t>0x1f877654f3c926ae529b6ddd3c7171b2d13a4a8d5ebf0feacc94d11ce8030cd0</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0xFD3Cd99B8d9ff9F970d873FD51Db34a241440516</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2170,22 +2162,22 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>4.99998</t>
+          <t>137.93997</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.6963</t>
+          <t>1.8975</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Brasileiro Serie B</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2195,27 +2187,27 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>CRB vs Vila Nova GO</t>
+          <t>Atletico Goianiense vs Operario PR</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Vila Nova GO</t>
+          <t>Operario PR</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x164012f3264d9ee546eec79c1f187343794314881d9822a8fe97501455cef745</t>
+          <t>0xc8ef5bb61583039e96277733cf10bf29a1a696cbdd90f2cb2bccfce1f6069793</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>L19549036</t>
+          <t>L19548984</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2240,7 +2232,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1785192506</t>
+          <t>1785192985</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2250,7 +2242,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>7.1813</t>
+          <t>153.69356</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2267,12 +2259,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0xe710e0c0376a72f95ca778f9e5f3a8399edb9a229d58a6de28041cab6ca46ebc</t>
+          <t>0x6430a839f73026cc87b0d5a0b70654fed87b780609d9d10323dbb2e3d5981d2f</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3Cd99B8d9ff9F970d873FD51Db34a241440516</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2282,22 +2274,22 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>52.85</t>
+          <t>4.99998</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>1.6963</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Operario PR</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2307,27 +2299,27 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Atletico Goianiense vs Operario PR</t>
+          <t>CRB vs Vila Nova GO</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Operario PR</t>
+          <t>Vila Nova GO</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x009d97ace951d42df767e4f8051070c4ae71bc57b68e13d8724fbd523b67056f</t>
+          <t>0x164012f3264d9ee546eec79c1f187343794314881d9822a8fe97501455cef745</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>L19548984</t>
+          <t>L19549036</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2352,7 +2344,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1785191996</t>
+          <t>1785192506</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2362,7 +2354,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>587.222222</t>
+          <t>7.1813</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2379,7 +2371,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x2dd6170d0bb75ad4506c6e6e7d66349c95078c6af465ead37ce9752e5b0c998b</t>
+          <t>0xe710e0c0376a72f95ca778f9e5f3a8399edb9a229d58a6de28041cab6ca46ebc</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2387,28 +2379,36 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>66.90021</t>
+          <t>52.85</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.1113</t>
+          <t>1.09</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Operario PR</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
           <t>Brasileiro Serie B</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Brasileiro Serie B</t>
-        </is>
-      </c>
       <c r="I19" t="inlineStr">
         <is>
           <t>Atletico Goianiense vs Operario PR</t>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0xc8ef5bb61583039e96277733cf10bf29a1a696cbdd90f2cb2bccfce1f6069793</t>
+          <t>0x009d97ace951d42df767e4f8051070c4ae71bc57b68e13d8724fbd523b67056f</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2456,7 +2456,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1785191995</t>
+          <t>1785191996</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>601.350202</t>
+          <t>587.222222</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2483,39 +2483,31 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x60f51d4feeddc57e7ad54ec8e925642a90b92e40913e7bf9f7d10e2ab8f78f00</t>
+          <t>0x2dd6170d0bb75ad4506c6e6e7d66349c95078c6af465ead37ce9752e5b0c998b</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>66.90021</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.1113</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Under/Over (4.5)</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Over 4.5</t>
-        </is>
-      </c>
+          <t>Brasileiro Serie B</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -2538,7 +2530,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0x563c254290f2bca3349399de0f58716204283212536d68ecebbda660883e8955</t>
+          <t>0xc8ef5bb61583039e96277733cf10bf29a1a696cbdd90f2cb2bccfce1f6069793</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2568,7 +2560,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1785191869</t>
+          <t>1785191995</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2578,7 +2570,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>6.166667</t>
+          <t>601.350202</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2595,12 +2587,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0xe778363b4557273dd14de4337865dd189b21126e8ba81bee67f5eb20692ac1c0</t>
+          <t>0x60f51d4feeddc57e7ad54ec8e925642a90b92e40913e7bf9f7d10e2ab8f78f00</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2610,22 +2602,22 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>123.99</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.5012</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>Under/Over (4.5)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>CRB -0.5</t>
+          <t>Over 4.5</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2635,27 +2627,27 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>CRB vs Vila Nova GO</t>
+          <t>Atletico Goianiense vs Operario PR</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Vila Nova GO</t>
+          <t>Operario PR</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0xa9304c5be90462f067ad52886159b64d91c9a8468c0aff2fafb714ca682b39e0</t>
+          <t>0x563c254290f2bca3349399de0f58716204283212536d68ecebbda660883e8955</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>L19549036</t>
+          <t>L19548984</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2680,7 +2672,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1785191301</t>
+          <t>1785191869</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2690,7 +2682,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>247.361596</t>
+          <t>6.166667</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2707,31 +2699,39 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x76badc2285724881b122bebddf6b9e6c4c3cf3e4a05d3690b012b1cc148fbfde</t>
+          <t>0xe778363b4557273dd14de4337865dd189b21126e8ba81bee67f5eb20692ac1c0</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr"/>
+          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>599.87913</t>
+          <t>123.99</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.7637</t>
+          <t>1.5012</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr"/>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>CRB -0.5</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -2754,7 +2754,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0xccd12abb617dfc61183a060a3ae6528413e3d3f34e761b9f0acc3557c868245d</t>
+          <t>0xa9304c5be90462f067ad52886159b64d91c9a8468c0aff2fafb714ca682b39e0</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2784,7 +2784,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1785191158</t>
+          <t>1785191301</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>785.439123</t>
+          <t>247.361596</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2811,7 +2811,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x91ddeba03b208be248ba41a4881c3c4c7d0715d371e6263f2e0b4290cec16b1b</t>
+          <t>0x76badc2285724881b122bebddf6b9e6c4c3cf3e4a05d3690b012b1cc148fbfde</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2822,17 +2822,17 @@
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>49.90293</t>
+          <t>599.87913</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.3813</t>
+          <t>1.7637</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
@@ -2843,27 +2843,27 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE vs Cuiaba</t>
+          <t>CRB vs Vila Nova GO</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>Vila Nova GO</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0xd514accb2f809d1aa051e761e590fdb70d8359c432892ab528533d38968148e5</t>
+          <t>0xccd12abb617dfc61183a060a3ae6528413e3d3f34e761b9f0acc3557c868245d</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>L19549019</t>
+          <t>L19549036</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2888,7 +2888,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1785191085</t>
+          <t>1785191158</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2898,7 +2898,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>130.892931</t>
+          <t>785.439123</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2915,7 +2915,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0x5d9ee4415a1e3226e79c82a0ad8402f41a775d58348c69deb79a0f1f8f6795d6</t>
+          <t>0x91ddeba03b208be248ba41a4881c3c4c7d0715d371e6263f2e0b4290cec16b1b</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2926,17 +2926,17 @@
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
-          <t>31.75047</t>
+          <t>49.90293</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.5275</t>
+          <t>1.3813</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
@@ -2962,7 +2962,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0x54bd394d0f69cdedbefc7e393cac97bba562ca5d9c533011ea99d1ec4c012a2b</t>
+          <t>0xd514accb2f809d1aa051e761e590fdb70d8359c432892ab528533d38968148e5</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>60.190464</t>
+          <t>130.892931</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3019,7 +3019,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x057b9dc707d522517e9353e2008a44693bea8ac1ca696f3200b57eb2c82453bb</t>
+          <t>0x5d9ee4415a1e3226e79c82a0ad8402f41a775d58348c69deb79a0f1f8f6795d6</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3030,17 +3030,17 @@
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>23.10284</t>
+          <t>31.75047</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.3838</t>
+          <t>1.5275</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
@@ -3066,7 +3066,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0xd514accb2f809d1aa051e761e590fdb70d8359c432892ab528533d38968148e5</t>
+          <t>0x54bd394d0f69cdedbefc7e393cac97bba562ca5d9c533011ea99d1ec4c012a2b</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -3106,7 +3106,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>60.20284</t>
+          <t>60.190464</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3123,28 +3123,28 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0x6ec8571db656bf4ace15e41ee9319395aaf946ddda18f3df168f286a1a1bb4ff</t>
+          <t>0x057b9dc707d522517e9353e2008a44693bea8ac1ca696f3200b57eb2c82453bb</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>8.99</t>
+          <t>23.10284</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.2463</t>
+          <t>1.3838</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
@@ -3170,7 +3170,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0x7f2fb02659d83b890cfe18154671039eb222ef3a24f76c4dc7c26b4868ea21bf</t>
+          <t>0xd514accb2f809d1aa051e761e590fdb70d8359c432892ab528533d38968148e5</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3200,7 +3200,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1785190227</t>
+          <t>1785191085</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>36.507614</t>
+          <t>60.20284</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3227,28 +3227,28 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0xa9f26cf6e000e4922c2f38b67d28a2deda7559922560443baab526b4b0c61b73</t>
+          <t>0x6ec8571db656bf4ace15e41ee9319395aaf946ddda18f3df168f286a1a1bb4ff</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>46.73411</t>
+          <t>8.99</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.3313</t>
+          <t>1.2463</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Brasileiro Serie B</t>
+          <t>Asian Handicap (0.5)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
@@ -3259,27 +3259,27 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>CRB vs Vila Nova GO</t>
+          <t>Sport Club Recife PE vs Cuiaba</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Sport Club Recife PE</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Vila Nova GO</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0xd53171a74e0242d67f30a86b7aaa3d2b2cde7e733a1beb26cf0c703dbab1e0c6</t>
+          <t>0x7f2fb02659d83b890cfe18154671039eb222ef3a24f76c4dc7c26b4868ea21bf</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>L19549036</t>
+          <t>L19549019</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -3304,7 +3304,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1785189680</t>
+          <t>1785190227</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>141.084106</t>
+          <t>36.507614</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3331,7 +3331,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0x0e0907f0172fe7e0b1a15423f1c2ea46f221e75a91330b9fcd0210b43161dffc</t>
+          <t>0xa9f26cf6e000e4922c2f38b67d28a2deda7559922560443baab526b4b0c61b73</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3342,7 +3342,7 @@
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>70.48505</t>
+          <t>46.73411</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1785189678</t>
+          <t>1785189680</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>212.785057</t>
+          <t>141.084106</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3435,7 +3435,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0xd2e589ce8fd3d5a2041b18219e18e34205c142aa8a4e07e600978a682778f7dd</t>
+          <t>0x0e0907f0172fe7e0b1a15423f1c2ea46f221e75a91330b9fcd0210b43161dffc</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3443,31 +3443,23 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>16.03</t>
+          <t>70.48505</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.2662</t>
+          <t>1.3313</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>CRB -1</t>
-        </is>
-      </c>
+          <t>Brasileiro Serie B</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -3490,7 +3482,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0xb474c8115d11c43ca774879d23888594610a0050926049c5871c02ad70442828</t>
+          <t>0xd53171a74e0242d67f30a86b7aaa3d2b2cde7e733a1beb26cf0c703dbab1e0c6</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3520,7 +3512,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1785189440</t>
+          <t>1785189678</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3530,7 +3522,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>60.206573</t>
+          <t>212.785057</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3547,12 +3539,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0x7067e247051a48c87b2711f56e00831cc9cf38c00816148557da5dde43e0b18d</t>
+          <t>0xd2e589ce8fd3d5a2041b18219e18e34205c142aa8a4e07e600978a682778f7dd</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -3562,22 +3554,22 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>16.03</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.2312</t>
+          <t>1.2662</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>CRB -1</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -3587,27 +3579,27 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE vs Cuiaba</t>
+          <t>CRB vs Vila Nova GO</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>Vila Nova GO</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0xcbd93d924a25bfc5eed272e7eebb053f11cd7a088fbde08dafa66b1ccb19d6d2</t>
+          <t>0xb474c8115d11c43ca774879d23888594610a0050926049c5871c02ad70442828</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>L19549019</t>
+          <t>L19549036</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -3632,7 +3624,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1785188684</t>
+          <t>1785189440</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -3642,7 +3634,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>5.102703</t>
+          <t>60.206573</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3659,12 +3651,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0xfef3f05953c1b69da0cb3db16102cf296b132ec89570e3b07a5a0c924d4de594</t>
+          <t>0x7067e247051a48c87b2711f56e00831cc9cf38c00816148557da5dde43e0b18d</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -3674,22 +3666,22 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>15.88</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.2637</t>
+          <t>1.2312</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>CRB -1</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -3699,27 +3691,27 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>CRB vs Vila Nova GO</t>
+          <t>Sport Club Recife PE vs Cuiaba</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Sport Club Recife PE</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Vila Nova GO</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0xb474c8115d11c43ca774879d23888594610a0050926049c5871c02ad70442828</t>
+          <t>0xcbd93d924a25bfc5eed272e7eebb053f11cd7a088fbde08dafa66b1ccb19d6d2</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>L19549036</t>
+          <t>L19549019</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -3744,7 +3736,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1785188472</t>
+          <t>1785188684</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -3754,7 +3746,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>60.208531</t>
+          <t>5.102703</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3771,12 +3763,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0xfc5ef9a86c99fd1897abcd8e09889e7009f6384950e112b87a199335cb42db0a</t>
+          <t>0xfef3f05953c1b69da0cb3db16102cf296b132ec89570e3b07a5a0c924d4de594</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0x155C76202e45BE70c50bfeD7eAeA3B98e7716Ff7</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -3786,22 +3778,22 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15.88</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.3362</t>
+          <t>1.2637</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>CRB -1</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -3811,27 +3803,27 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE vs Cuiaba</t>
+          <t>CRB vs Vila Nova GO</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Sport Club Recife PE</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>Vila Nova GO</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0x8534ef5ad4f16561c7b4121752a6a7b2095d700e69722155902e66e998ff0f55</t>
+          <t>0xb474c8115d11c43ca774879d23888594610a0050926049c5871c02ad70442828</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>L19549019</t>
+          <t>L19549036</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -3856,7 +3848,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1785188354</t>
+          <t>1785188472</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3866,7 +3858,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>2.973978</t>
+          <t>60.208531</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3883,7 +3875,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0x70f793d7639e9071725b67e5d59645a0ce3151b32e612fa9a3861ddf68c40caa</t>
+          <t>0xfc5ef9a86c99fd1897abcd8e09889e7009f6384950e112b87a199335cb42db0a</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3995,12 +3987,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0x0b1b494627a939fced86315d5bf47db8fed3489803145f8581ed0e6feeb9778a</t>
+          <t>0x70f793d7639e9071725b67e5d59645a0ce3151b32e612fa9a3861ddf68c40caa</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x155C76202e45BE70c50bfeD7eAeA3B98e7716Ff7</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -4010,12 +4002,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>10.48681</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.4663</t>
+          <t>1.3362</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4025,7 +4017,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -4035,27 +4027,27 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Atletico Goianiense vs Operario PR</t>
+          <t>Sport Club Recife PE vs Cuiaba</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>Sport Club Recife PE</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Operario PR</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0x12cd5e193bc63289c7fafbc19303377b9c4255fccb0ecd5d041453d8fa88faff</t>
+          <t>0x8534ef5ad4f16561c7b4121752a6a7b2095d700e69722155902e66e998ff0f55</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>L19548984</t>
+          <t>L19549019</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -4080,7 +4072,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1785188344</t>
+          <t>1785188354</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -4090,7 +4082,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>22.491818</t>
+          <t>2.973978</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4107,7 +4099,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0xed0c6b1bbdd31be7427b5ffe7a264e0c13f41925ed28604921031109f2b0cefa</t>
+          <t>0x0b1b494627a939fced86315d5bf47db8fed3489803145f8581ed0e6feeb9778a</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4122,12 +4114,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>10.12</t>
+          <t>10.48681</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.4575</t>
+          <t>1.4663</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4192,7 +4184,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1785188299</t>
+          <t>1785188344</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4202,7 +4194,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>22.120219</t>
+          <t>22.491818</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4219,12 +4211,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0x91583f323297c551497af92aef42c1fbe90007daddf717ff653e1533369fe9d5</t>
+          <t>0xed0c6b1bbdd31be7427b5ffe7a264e0c13f41925ed28604921031109f2b0cefa</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -4234,22 +4226,22 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>16.03</t>
+          <t>10.12</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.2662</t>
+          <t>1.4575</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>CRB -1</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -4259,27 +4251,27 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>CRB vs Vila Nova GO</t>
+          <t>Atletico Goianiense vs Operario PR</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Vila Nova GO</t>
+          <t>Operario PR</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0xb474c8115d11c43ca774879d23888594610a0050926049c5871c02ad70442828</t>
+          <t>0x12cd5e193bc63289c7fafbc19303377b9c4255fccb0ecd5d041453d8fa88faff</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>L19549036</t>
+          <t>L19548984</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -4304,7 +4296,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1785188207</t>
+          <t>1785188299</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4314,7 +4306,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>60.206573</t>
+          <t>22.120219</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4331,23 +4323,27 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0x093df5c9b7626116d81288cd377d306eb5151086a71a2bd3951894182b307e34</t>
+          <t>0x91583f323297c551497af92aef42c1fbe90007daddf717ff653e1533369fe9d5</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0xFBd63A3Adf898EfFf1e5A017f98756dC760eBfb8</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>49.4</t>
+          <t>16.03</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.7412</t>
+          <t>1.2662</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -4355,7 +4351,11 @@
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>CRB -1</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
@@ -4408,7 +4408,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1785187880</t>
+          <t>1785188207</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -4418,7 +4418,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>66.644182</t>
+          <t>60.206573</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4435,110 +4435,214 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>0x093df5c9b7626116d81288cd377d306eb5151086a71a2bd3951894182b307e34</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>0xFBd63A3Adf898EfFf1e5A017f98756dC760eBfb8</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>49.4</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>1.7412</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Brasileiro Serie B</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>CRB vs Vila Nova GO</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Vila Nova GO</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>0xb474c8115d11c43ca774879d23888594610a0050926049c5871c02ad70442828</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>L19549036</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>1785187880</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>1785191400</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>66.644182</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>0xf90085256f332e2273158e6e0b53485388f9d9e64670022d5b32ffc4aed4b545</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>0xFBd63A3Adf898EfFf1e5A017f98756dC760eBfb8</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
         <is>
           <t>134.62107</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>1.285</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>CRB -1</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>Brasileiro Serie B</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>CRB vs Vila Nova GO</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="J39" t="inlineStr">
         <is>
           <t>CRB</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t>Vila Nova GO</t>
         </is>
       </c>
-      <c r="L38" t="inlineStr">
+      <c r="L39" t="inlineStr">
         <is>
           <t>0xb474c8115d11c43ca774879d23888594610a0050926049c5871c02ad70442828</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr">
+      <c r="M39" t="inlineStr">
         <is>
           <t>L19549036</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O38" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P38" t="inlineStr">
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q38" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R38" t="inlineStr">
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
         <is>
           <t>1785187268</t>
         </is>
       </c>
-      <c r="S38" t="inlineStr">
+      <c r="S39" t="inlineStr">
         <is>
           <t>1785191400</t>
         </is>
       </c>
-      <c r="T38" t="inlineStr">
+      <c r="T39" t="inlineStr">
         <is>
           <t>472.354632</t>
         </is>
       </c>
-      <c r="U38" t="inlineStr">
+      <c r="U39" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V38" t="inlineStr">
+      <c r="V39" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>